<commit_message>
Completar la tabla por categoria del resumen con Medio, Bajo y Muy bajo
La tabla solo mostraba Extremo, Alto y Total, de modo que las columnas no
sumaban el total de la fila y los riesgos de nivel medio o bajo quedaban
invisibles por categoria. Ahora incluye los cinco niveles y cada fila cuadra
con su total.

Para que el texto de las tablas superiores conserve su ancho, la columna E deja
de ser la columna ancha y esas celdas se fusionan de E a H.

Se incluye tambien la copia del archivo diligenciada por el usuario
(Version_Rapida_3) con la misma correccion aplicada sobre su estructura, que
difiere de la generada: hojas renombradas, encabezado en la fila 1 y sin las
columnas de consecuencia y de detalle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DjaDU3QHWLpSnaydDxYzf7
</commit_message>
<xml_diff>
--- a/Checklist_Riesgos_CEDI_Version_Rapida.xlsx
+++ b/Checklist_Riesgos_CEDI_Version_Rapida.xlsx
@@ -7794,14 +7794,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7847,6 +7850,9 @@
           <t>Frecuencia mínima que exige</t>
         </is>
       </c>
+      <c r="F5" s="43" t="n"/>
+      <c r="G5" s="43" t="n"/>
+      <c r="H5" s="30" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="31" t="inlineStr">
@@ -7867,6 +7873,9 @@
           <t>Diaria o por turno + inspección formal semanal</t>
         </is>
       </c>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="33" t="inlineStr">
@@ -7887,6 +7896,9 @@
           <t>Semanal + inspección formal mensual</t>
         </is>
       </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="34" t="inlineStr">
@@ -7907,6 +7919,9 @@
           <t>Mensual (operativo) o trimestral (estructural)</t>
         </is>
       </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="35" t="inlineStr">
@@ -7927,6 +7942,9 @@
           <t>Semestral</t>
         </is>
       </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="36" t="inlineStr">
@@ -7947,6 +7965,9 @@
           <t>Anual</t>
         </is>
       </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="46" t="inlineStr">
@@ -7990,6 +8011,9 @@
           <t>Qué hacer</t>
         </is>
       </c>
+      <c r="F14" s="43" t="n"/>
+      <c r="G14" s="43" t="n"/>
+      <c r="H14" s="30" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="10" t="inlineStr">
@@ -8010,6 +8034,9 @@
           <t>Mantener el control y conservar su evidencia</t>
         </is>
       </c>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="10" t="inlineStr">
@@ -8030,6 +8057,9 @@
           <t>Cerrar la brecha dentro del plazo del nivel de riesgo</t>
         </is>
       </c>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="10" t="inlineStr">
@@ -8050,6 +8080,9 @@
           <t>Pasa al plan de acción con responsable y fecha</t>
         </is>
       </c>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="10" t="inlineStr">
@@ -8070,6 +8103,9 @@
           <t>Dejar registrado por qué no aplica</t>
         </is>
       </c>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="10" t="inlineStr">
@@ -8090,6 +8126,9 @@
           <t>Pendiente de verificar en campo</t>
         </is>
       </c>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="46" t="inlineStr">
@@ -8151,6 +8190,21 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Muy bajo</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -8170,6 +8224,18 @@
         <v>7</v>
       </c>
       <c r="E25" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B25,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B25,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B25,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B25)</f>
         <v>7</v>
       </c>
@@ -8189,6 +8255,18 @@
         <v>5</v>
       </c>
       <c r="E26" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B26,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B26,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B26,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B26)</f>
         <v>7</v>
       </c>
@@ -8208,6 +8286,18 @@
         <v>1</v>
       </c>
       <c r="E27" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B27,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B27,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B27,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B27)</f>
         <v>3</v>
       </c>
@@ -8227,6 +8317,18 @@
         <v>4</v>
       </c>
       <c r="E28" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B28,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B28,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B28,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B28)</f>
         <v>4</v>
       </c>
@@ -8246,6 +8348,18 @@
         <v>4</v>
       </c>
       <c r="E29" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B29,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B29,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B29,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B29)</f>
         <v>5</v>
       </c>
@@ -8265,6 +8379,18 @@
         <v>4</v>
       </c>
       <c r="E30" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B30,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>1</v>
+      </c>
+      <c r="F30" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B30,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B30,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B30)</f>
         <v>7</v>
       </c>
@@ -8284,6 +8410,18 @@
         <v>1</v>
       </c>
       <c r="E31" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B31,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>2</v>
+      </c>
+      <c r="F31" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B31,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B31,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B31)</f>
         <v>3</v>
       </c>
@@ -8303,6 +8441,18 @@
         <v>2</v>
       </c>
       <c r="E32" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B32,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B32,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B32,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B32)</f>
         <v>2</v>
       </c>
@@ -8322,6 +8472,18 @@
         <v>2</v>
       </c>
       <c r="E33" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B33,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>2</v>
+      </c>
+      <c r="F33" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B33,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B33,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B33)</f>
         <v>4</v>
       </c>
@@ -8341,6 +8503,18 @@
         <v>2</v>
       </c>
       <c r="E34" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B34,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B34,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B34,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B34)</f>
         <v>2</v>
       </c>
@@ -8360,6 +8534,18 @@
         <v>4</v>
       </c>
       <c r="E35" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B35,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>1</v>
+      </c>
+      <c r="F35" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B35,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B35,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B35)</f>
         <v>5</v>
       </c>
@@ -8379,6 +8565,18 @@
         <v>5</v>
       </c>
       <c r="E36" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B36,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B36,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B36,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B36)</f>
         <v>5</v>
       </c>
@@ -8398,6 +8596,18 @@
         <v>1</v>
       </c>
       <c r="E37" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B37,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>1</v>
+      </c>
+      <c r="F37" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B37,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B37,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B37)</f>
         <v>2</v>
       </c>
@@ -8417,6 +8627,18 @@
         <v>2</v>
       </c>
       <c r="E38" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B38,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B38,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B38,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B38)</f>
         <v>2</v>
       </c>
@@ -8436,15 +8658,41 @@
         <v>2</v>
       </c>
       <c r="E39" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B39,'2. Matriz rápida'!$I$5:$I$66,"Medio")</f>
+        <v>2</v>
+      </c>
+      <c r="F39" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B39,'2. Matriz rápida'!$I$5:$I$66,"Bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="8">
+        <f>COUNTIFS('2. Matriz rápida'!$B$5:$B$66,$B39,'2. Matriz rápida'!$I$5:$I$66,"Muy bajo")</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="10">
         <f>COUNTIF('2. Matriz rápida'!$B$5:$B$66,$B39)</f>
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A23:E23"/>
+  <mergeCells count="17">
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="E17:H17"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="E18:H18"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E20:H20"/>
+    <mergeCell ref="E16:H16"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E15:H15"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="E5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>